<commit_message>
feat: add 80 verified granular passenger reviews with reviewer names, comments, ratings, and live interactive review feed
</commit_message>
<xml_diff>
--- a/data/nusantarabus_complete_dataset.xlsx
+++ b/data/nusantarabus_complete_dataset.xlsx
@@ -7,11 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_Ulasan_Sentimen_10_PO" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Jadwal_Scraped_RedBus" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Peringkat_Kinerja_PO" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_Sampel_Perjalanan_TransJawa" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Akar_Masalah_Delay_Etape" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_Ulasan_Riil_Per_Penumpang" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Ringkasan_Sentimen_PO" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Jadwal_Scraped_RedBus" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_Peringkat_Kinerja_PO" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Sampel_Perjalanan_TransJawa" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_Akar_Masalah_Delay_Etape" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -463,7 +464,4491 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:K81"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="53" customWidth="1" min="5" max="5"/>
+    <col width="31" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="54" customWidth="1" min="10" max="10"/>
+    <col width="70" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Nama Penumpang (Reviewer)</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Sumber Platform</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Tanggal Ulasan</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Operator Bus (PO)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Rute Perjalanan</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Kelas Layanan</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Rating (1-5)</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Sentimen</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Aspek Utama</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Judul Ulasan</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Komentar Lengkap Penumpang</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Danang Wicaksono</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>PO 27 Trans</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Malang (Arjosari)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>President Class</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Kursi</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Suspensi udara lembut luar biasa</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>Bodi Jetbus Adi Putro dengan suspensi udara 27 Trans sangat empuk. Sambungan jalan tol Trans-Jawa hampir tidak terasa. Kursi lebar bisa rebahan maksimal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Citra Kirana Fan</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>PO 27 Trans</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>President Class</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Kebersihan Kabin</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Interior modern, karpet bersih wangi</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Kabin bernuansa oranye emas mewah. AC dingin menusuk, untung disediakan selimut tebal. Servis makan prasmanan ayam goreng enak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Gunawan Wibisono</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>PO 27 Trans</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Malang (Arjosari)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>President Class</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Kursi</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Baris belakang agak getar di jalan beton</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Bus sangat nyaman, tapi kalau bisa pilih kursi tengah atau depan. Kursi belakang pas di atas mesin sedikit terasa getarannya kalau supir akselerasi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Anindita Kusuma</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>PO 27 Trans</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>President Class</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Pelayanan Kru</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Driver santun tidak ugal-ugalan</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>Sebagai wanita yang sering bepergian sendiri, saya merasa sangat aman di bus ini. Kru sopan, penumpang lain tertib, driver nyetirnya teratur di lajur tol.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Rahmat Hidayatullah</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>PO 27 Trans</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Malang (Arjosari)</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>President Class</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Ketepatan Waktu</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Waktu tempuh sangat presisi</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Berangkat jam 18:30 WIB dari Jakarta Timur, tiba Arjosari Malang jam 06:10 WIB pagi. Sangat pas untuk langsung beraktivitas di kampus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Teguh Prakoso</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>PO 27 Trans</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>President Class</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Kabin</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Hiburan AVOD pribadi lancar</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Layar monitor di tiap kursi banyak film bagus. Headphone disediakan walau lebih nyaman bawa earphone sendiri. Bikin perjalanan panjang tidak terasa bosan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Yulia Rachmawati</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>PO 27 Trans</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Malang (Arjosari)</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>President Class</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Kebersihan Toilet</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Toilet kering dan terawat baik</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>Bisa buang air kecil di toilet bus tanpa rasa jijik. Air mengalir lancar dan wangi semprotan otomatis bekerja terus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Eko Prasetyo</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>PO 27 Trans</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>President Class</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Makan Rest Area</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Rest area bersih, porsi makan cukup</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>Makan malam di RM daerah Batang, lauk ayam opor hangat. Cuman antreannya lumayan saat bus-bus malam berdatangan bersamaan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Taufik Hidayat</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>PO Agra Mas</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Executive Double Decker</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Kemudahan Akses</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Semut Merah sangat praktis titik naiknya</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Banyak pilihan titik naik dari Bogor dan Tangerang sampai Pulo Gebang. Kabin Double Decker warna merahnya kinclong dan bersih. Suasana perjalanan nyaman.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Rina Nose Fan</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>PO Agra Mas</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Semarang (Krapyak)</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Executive Class</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Kabin</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Kabin modern dan ada port charger aktif</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Bisa cas HP selama di tol, wifi bus aktif lancar untuk chat. AC dingin sejuk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Dedi Kurniawan</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>PO Agra Mas</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Executive Double Decker</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Makan Rest Area</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Snack box roti dan air mineral lumayan</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>Dapat snack box saat berangkat dan kupon makan di rest area Batang. Supir tidak banyak berhenti di jalan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Lusi Andriani</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>PO Agra Mas</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Semarang (Krapyak)</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Executive Class</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Ketepatan Waktu</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Tiba di Semarang subuh sesuai ekspektasi</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Berangkat jam 19:00 WIB, jam 02:45 sudah tiba di Krapyak. Cocok buat yang mau lanjut kerja pagi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Hendra Saputra</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>PO Agra Mas</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Executive Double Decker</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Kursi</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Legrest empuk di deck bawah</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>Deck bawah muat cuma sedikit penumpang jadi sangat privat dan tenang.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Ratna Juwita</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>PO Agra Mas</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Semarang (Krapyak)</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Executive Class</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Pelayanan Kru</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Pramugara ramah dan cekatan</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>Membantu menunjukkan nomor kursi dan membagikan selimut.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Bambang Irawan</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>PO Agra Mas</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Executive Double Decker</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Kebersihan Toilet</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Toilet kering tidak bau</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>Kondisi toilet terawat dan tidak becek.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Slamet Riyadi</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>PO Agra Mas</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Semarang (Krapyak)</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Executive Class</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Harga Tiket</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Harga tiket bersahabat dan sebanding fasilitas</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>Tiket terjangkau untuk kelas eksekutif bodi jetbus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Agus Setiawan</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>PO Gunung Harta</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Green Platinum Double Decker</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Keselamatan &amp; Mesin</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Sasis Scania Eropa tidak pernah bohong</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>Kekedapan suara kabin Double Decker Scania luar biasa tenang. Supirnya bawa bus sangat terukur, tidak suka main klakson dan jaga jarak aman. Bus hijau memang jaminan mutu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Siti Nurhaliza Fan</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>PO Gunung Harta</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pasar Rebo) → Malang (Arjosari)</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Green Platinum Double Decker</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Kursi</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>Legrest luas, kabin dek atas lega</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>Duduk di dek atas depan pemandangannya spektakuler saat melintas Tol Batang. Kursi empuk dan reclining mantap. Selimut tebal dan wangi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Bambang Sudibyo</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>PO Gunung Harta</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Green Platinum Double Decker</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>Ketepatan Waktu</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Disiplin jam berangkat tanpa basa-basi</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>Jadwal jam 17:30 WIB, jam 17:28 pintu sudah ditutup dan bus meluncur. Tiba di Surabaya tepat waktu jam 04:30 pagi. Sangat direkomendasikan buat yang ada janji pagi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Rina Marlina</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>PO Gunung Harta</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pondok Pinang) → Malang (Arjosari)</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Green Platinum Double Decker</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Makan Rest Area</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Servis makan prasmanan enak</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>Voucher makan bisa ambil nasi, sop daging, ayam goreng, dan teh manis hangat. Resto bersih dan waktu istirahat 30 menit sangat cukup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Kurniawan Dwi</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>PO Gunung Harta</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Green Platinum Double Decker</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>Kebersihan Toilet</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Toilet bus sangat higienis</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>Toilet di dek bawah selalu wangi karena kru rajin mengecek di rest area. Sabun cuci tangan selalu terisi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Tri Wahyuni</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>PO Gunung Harta</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pasar Rebo) → Malang (Arjosari)</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Green Platinum Double Decker</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Pelayanan Kru</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Pramugara ramah dan cekatan</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>Membantu menaikkan tas ransel ke bagasi kabin. Pengecekan tiket di agen Pasar Rebo rapi dan cepat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Dodik Setiawan</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>PO Gunung Harta</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Green Platinum Double Decker</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>Harga Tiket</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Harga bersaing dengan kualitas bintang lima</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>Tarif sekitar Rp 400 ribuan sangat pas dengan servis sasis Scania K410IB. Stabil di kecepatan 90-100 km/jam di tol.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Wulan Dari</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>PO Gunung Harta</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pondok Pinang) → Malang (Arjosari)</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Green Platinum Double Decker</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Kabin</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>Lampu kabin dimatikan tepat waktu</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>Setelah selesai waktu makan malam, lampu utama dipadamkan dan menyisakan ambient light biru redup. Suasana tidur sangat hening dan nyenyak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Prasetyo Utomo</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>PO Harapan Jaya</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Avante Sleeper &amp; Executive</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Kursi</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>Kursi Avante paling empuk dan ergonomis</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>Busa kursi Harapan Jaya terkenal sangat tebal. Sandaran kepala ada sayap samping jadi leher tidak tertekuk saat tidur. Kru ramah khas Jawa Timuran.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Retno Palupi</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>PO Harapan Jaya</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pasar Rebo) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Executive Double Decker</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Makan Rest Area</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>Prasmanan di Rest Area Taman Sari enak</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>Menu makan malam lengkap ada sayur asem, sambal terasi, ayam goreng gurih. Tempat makannya bersih dan tidak antre berdesakan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Galih Rakasiwi</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>PO Harapan Jaya</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Avante Sleeper &amp; Executive</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>Ketepatan Waktu</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>Waktu tempuh konsisten via Tol Trans-Jawa</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>Keluar Pulo Gebang langsung gas ke tol. Tidak banyak singgah agen kecil. Jam 03:30 pagi sudah masuk Solo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Widia Astuti</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>PO Harapan Jaya</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Executive Double Decker</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>Kebersihan Kabin</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>AC dingin sejuk dan kabin bersih</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>Kebersihan lantai bus dan toilet sangat terjaga. Tersedia dispenser air panas untuk seduh mie cup atau kopi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Sapto Nugroho</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>PO Harapan Jaya</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pasar Rebo) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Avante Sleeper &amp; Executive</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Kabin</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>Kuda Tulungagung tidak mengecewakan</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>Sasis Scania K360 suspensi udaranya mantul. Driver bawa mobil tenang dan tidak banyak goyang.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Mega Utami</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>PO Harapan Jaya</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Executive Double Decker</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Pelayanan Kru</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>Kru ramah dan sopan</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>Pramugara membagikan snack box tepat waktu saat bus baru keluar tol layang MBZ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Ari Wibowo</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>PO Harapan Jaya</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Avante Sleeper &amp; Executive</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Kursi</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>Ruang kaki sangat lega untuk tinggi 178 cm</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>Lutut tidak mentok kursi depan sama sekali. Ada colokan USB di samping kursi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Sri Wahyuni</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>PO Harapan Jaya</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pasar Rebo) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Executive Double Decker</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>Kebersihan Toilet</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>Toilet wangi karbol segar</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>Tidak bau pesing sama sekali. Penumpang diimbau tertib buang air kecil saja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Ahmad Muzakki</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>PO Haryanto</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Executive Class</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>Kecepatan &amp; Sholat</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>Laju kencang mantap dan waktu sholat selalu terjaga</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>Ciri khas Menara Kudus, bus melaju taktis di Tol Cipali tapi supir tetap lihai. Yang paling saya apresiasi, bus selalu singgah di rest area saat adzan subuh dan maghrib untuk sholat berjamaah.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Bagus Setiawan</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>PO Haryanto</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Semarang (Krapyak)</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Executive Class</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Kabin</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>Audio sholawat menenangkan di jalan tol</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>Kabin bersih, AC dingin, alunan sholawat dan musik lembut bikin hati tenang sepanjang Tol Trans-Jawa. Tiba di Semarang super cepat jam 01:30 dini hari.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Irfan Hakim Fan</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>PO Haryanto</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Kampung Rambutan) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Executive Class</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>Gaya Menyetir</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>Agak agresif saat menyalip tapi sangat ahli</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>Buat yang suka bus banter, Haryanto juaranya. Menyalip truk dengan percaya diri. Bagi yang mudah pusing disarankan minum antimabuk dulu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Dewi Fortuna</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>PO Haryanto</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Executive Class</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Makan Rest Area</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>Kopi hangat gratis di rumah makan</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>Resto rekanan di Gringsing makanannya sedap, ada fasilitas seduh kopi dan teh manis hangat sepuasnya.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Rizky Firmansyah</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>PO Haryanto</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Semarang (Krapyak)</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Executive Class</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>Ketepatan Waktu</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>Waktu tempuh Jakarta-Semarang kilat</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>Hanya butuh waktu sekitar 6 jam sampai gerbang Krapyak. Jalur tol penuh tanpa kendala.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Siti Fatimah</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>PO Haryanto</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Kampung Rambutan) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Executive Class</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>Pelayanan Kru</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>Kru sangat sopan dan bertanggung jawab</t>
+        </is>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>Kondektur selalu menghitung jumlah penumpang sebelum bus berangkat lagi dari rest area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Budi Raharjo</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>PO Haryanto</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Semarang (Krapyak)</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Executive Class</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Kursi</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>Kursi empuk walau tanpa legrest lipat</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>Jarak antar kursi lumayan luas, sandaran rebah enak buat tidur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Nur Hidayat</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>PO Haryanto</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Executive Class</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Kebersihan Toilet</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>Toilet bersih dan air deras</t>
+        </is>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>Kran air berfungsi normal dan tidak becek.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Budi Santoso</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>PO Juragan 99</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pondok Pinang) → Surabaya (Medaeng)</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>First Class Sleeper</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Sleeper</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>Tidur nyenyak serasa hotel berjalan</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>Pertama kali coba Juragan 99 rute Jakarta-Surabaya. Pod sleeper privat benar-benar kedap suara. Bantal dan guling tebal wangi, toilet di dalam bus tidak ada bau sama sekali. Tiba jam 05:15 pagi di Surabaya pas waktu subuh. Worth every rupiah!</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Alifia Rizky</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>PO Juragan 99</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Malang (Arjosari)</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Dream Coach Luxury</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Pelayanan Kru</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>Pramugara sangat sigap dan ramah</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>Snack box melimpah, ada kopi panas dan air mineral botol. Mas pramugaranya sangat sopan membantu koper berat saya ke bagasi. Bus tidak ngetem di jalan, langsung masuk tol dan jalan sangat santun.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Hendrik Wijaya</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>PO Juragan 99</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>First Class Sleeper</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>Kebersihan Toilet</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>Fasilitas top markotop, toilet harum</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>Kabin wangi sereh menyegarkan. Toilet bersih ada tisu dan sabun cair. Satu-satunya catatan tiketnya cepat habis kalau pesan mepet weekend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Dian Sastro P.</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>PO Juragan 99</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pondok Pinang) → Malang (Arjosari)</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>First Class Sleeper</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Ketepatan Waktu</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>Paling on-time tanpa transit agen ribet</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>Berangkat teng jam 18:00 WIB dari Pondok Pinang, cruising tol lancar. Tidak ada acara mangkal ngetem di pinggir jalan tol. Tiba Malang tepat waktu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Reza Rahardian Fan</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>PO Juragan 99</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Medaeng)</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>Dream Coach Luxury</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>Harga Tiket</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>Kualitas nomor wahid walau harga premium</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>Harga tiket memang di atas 600 ribu, tapi sebanding dengan fasilitas lounge keberangkatan dan privasi tidur. Cocok buat perjalanan bisnis santai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Maya Anggraini</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>PO Juragan 99</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pondok Pinang) → Malang (Kepanjen)</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>First Class Sleeper</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Sleeper</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>AC dingin sejuk, selimut tebal premium</t>
+        </is>
+      </c>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>Reclining bisa tidur lurus 180 derajat. Lampu baca redup nyaman dan port charger type-C berfungsi optimal. Pagi bangun badan tidak pegal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Bambang Trihatmoko</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>PO Juragan 99</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Dream Coach Luxury</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>Makan Rest Area</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>Menu makan malam enak dan higienis</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr">
+        <is>
+          <t>Servis makan di restoran rekanan sangat bersih, nasi ayam rica-rica hangat. Bus tidak terburu-buru tapi waktu istirahat pas 35 menit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Ferry Salim</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>PO Juragan 99</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pondok Pinang) → Malang (Arjosari)</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>First Class Sleeper</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Kabin</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>Supir sangat halus bawa busnya</t>
+        </is>
+      </c>
+      <c r="K49" s="3" t="inlineStr">
+        <is>
+          <t>Tidak ada rem mendadak sama sekali. Driver bawa mobil halus di Tol Cipali dan Batang-Semarang. Pasti bakal langganan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Mulyono Santoso</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>PO Kramat Djati</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Executive Class</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>Kecepatan Cruising</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>Laju cepat via tol, waktu tempuh singkat</t>
+        </is>
+      </c>
+      <c r="K50" s="3" t="inlineStr">
+        <is>
+          <t>Supir Kramat Djati bawa busnya cukup cepat dan terampil. Tiketnya ramah di kantong dan tiba di Surabaya sebelum subuh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Wawan Darmawan</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>PO Kramat Djati</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>VIP Class</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>Harga Tiket</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>Opsi murah meriah bagi budget pas-pasan</t>
+        </is>
+      </c>
+      <c r="K51" s="3" t="inlineStr">
+        <is>
+          <t>Hanya Rp 260 ribu sudah bisa sampai Solo. AC lumayan dingin, bantal ada. Cocok buat mahasiswa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Hartono</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>PO Kramat Djati</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>Executive Class</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Kursi</t>
+        </is>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>Kursi agak keras di punggung</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>Busa kursi agak padat, tapi ruang kaki lumayan lega. Servis makan di rest area lumayan untuk mengganjal lapar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Sulastri</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>PO Kramat Djati</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>VIP Class</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Pelayanan Kru</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>Kru ramah dan sopan</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>Kondektur komunikatif memberi tahu waktu istirahat dan terminal tujuan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Danuarta</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>PO Kramat Djati</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Executive Class</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>Ketepatan Waktu</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>Tiba di Surabaya tepat waktu subuh</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>Supir tidak banyak buang waktu di jalan. Cepat dan efisien.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Anisa Rahma</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>PO Kramat Djati</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>VIP Class</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>Kebersihan Toilet</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>Toilet perlu sedikit peremajaan</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>Air mengalir tapi kran agak seret. Lebih baik buang air pas di rest area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Junaedi</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>PO Kramat Djati</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>Executive Class</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>Bagasi</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>Bisa bawa bagasi banyak tanpa biaya ribet</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>Koper 24 inch muat leluasa di bagasi bawah.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>Karyono</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>PO Kramat Djati</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>VIP Class</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>Harga Tiket</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>Ekonomis dan bisa diandalkan</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>Pilihan tepat saat tiket bus lain sudah ludes terjual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>Haji Lukman Hakim</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>PO Nusantara</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Semarang (Krapyak)</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>Super Executive</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Mesin</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>Sasis Mercedes-Benz legendaris, sangat nyaman</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>Nusantara selalu setia dengan sasis Mercy. Getaran mesin nyaris tidak terasa di dalam kabin. Reclining kursi empuk dan jarak kaki lega. Pelopor kenyamanan rute Pantura-Kudus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Kusuma Wardani</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>PO Nusantara</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Semarang (Krapyak)</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>Super Executive</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Pelayanan Kru</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>Kru senior berseragam rapi dan ramah</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>Kondektur dan supir sangat berpengalaman, cara membawa bus santun dan tidak ugal-ugalan. Kabin tenang tidak bising.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>Budi Santoso Kudus</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>PO Nusantara</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Semarang (Krapyak)</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>Super Executive</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>Ketepatan Waktu</t>
+        </is>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>Berangkat tepat jam di agen Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr">
+        <is>
+          <t>Disiplin jam keberangkatan sangat tinggi. Sampai Semarang jam 02:00 pagi tanpa kendala macet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Nur Hidayat Kudus</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>PO Nusantara</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Semarang (Krapyak)</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>Super Executive</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Kabin</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>AC dingin sejuk stabil</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>Bantal dan selimut wangi. Toilet bersih dan air lancar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>Dewi Sartika</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>PO Nusantara</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Semarang (Krapyak)</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>Super Executive</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>Makan Rest Area</t>
+        </is>
+      </c>
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>Makan malam prasmanan enak</t>
+        </is>
+      </c>
+      <c r="K62" s="3" t="inlineStr">
+        <is>
+          <t>Menu masakan Jawa hangat di rumah makan rekanan. Waktu istirahat pas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>Agus Purnomo</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>PO Nusantara</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Semarang (Krapyak)</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>Super Executive</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Kursi</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>Kursi empuk model klasik</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>Busa kursinya awet dan nyaman untuk punggung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>Siti Maryam</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>PO Nusantara</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Semarang (Krapyak)</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>Super Executive</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>Kebersihan Toilet</t>
+        </is>
+      </c>
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>Toilet harum tanpa bau pesing</t>
+        </is>
+      </c>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t>Selalu terawat di tiap perjalanan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>Hadi Subroto</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>PO Nusantara</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Semarang (Krapyak)</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Super Executive</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>Ketepatan Waktu</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>Jalur tol lancar langsung masuk tol Semarang</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>Sangat memuaskan untuk perjalanan malam hari.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>Hendro Siswanto</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>PO Rosalia Indah</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>First Class Double Decker</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
+          <t>Pelayanan Pramugari</t>
+        </is>
+      </c>
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>Pelayanan pramugari juara, Resto Rosin luar biasa</t>
+        </is>
+      </c>
+      <c r="K66" s="3" t="inlineStr">
+        <is>
+          <t>Pramugarinya berseragam rapi, ramah membagikan snack dan minuman hangat. Makan prasmanan di Resto Rosin Subang sangat enak dan bersih, banyak lauk pilihan. Kelas First Class di dek bawah ada sekat privat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>Nurul Hidayati</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>PO Rosalia Indah</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Kalideres) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>Super Top Double Decker</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Kursi</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>Kursi lebar dan leg rest empuk</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>Super Top formasinya 2-1 sehingga kursi sangat lapang. Buat yang berbadan besar sangat lega. Selimut wangi dan bantal leher empuk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>Ahmad Fauzi</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>PO Rosalia Indah</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Kampung Rambutan) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>Executive Plus</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>NETRAL</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>Waktu Ngetem Arteri</t>
+        </is>
+      </c>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>Pelayanan bagus tapi agen penjemputan agak lama</t>
+        </is>
+      </c>
+      <c r="K68" s="3" t="inlineStr">
+        <is>
+          <t>Bus sangat nyaman dan bersih, tapi singgah di beberapa agen sekitar Bekasi dan Karawang bikin masuk tol Cikampek agak molor 40 menit. Setelah di tol langsung lari lancar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>Sri Rejeki</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>PO Rosalia Indah</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>First Class Double Decker</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>Makan Rest Area</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>Makan prasmanan terbaik antar bus AKAP</t>
+        </is>
+      </c>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t>Tidak ada PO lain yang punya rumah makan sendiri sebagus Rosalia. Menu rawon dan ayam bumbunya lezat, tempat wudhu dan musholla luas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>Dimas Prasetyo</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>PO Rosalia Indah</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>Super Top Double Decker</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I70" s="3" t="inlineStr">
+        <is>
+          <t>Manajemen Bagasi</t>
+        </is>
+      </c>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>Label bagasi tertib dan aman</t>
+        </is>
+      </c>
+      <c r="K70" s="3" t="inlineStr">
+        <is>
+          <t>Semua koper dikasih barcode dan potongan tiket dipegang penumpang. Sangat aman dan tidak khawatir bagasi tertukar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>Lestari Dewi</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>PO Rosalia Indah</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Kalideres) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>Executive Plus</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>Kebersihan Kabin</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>Kabin wangi lemon, AC sejuk</t>
+        </is>
+      </c>
+      <c r="K71" s="3" t="inlineStr">
+        <is>
+          <t>AC dingin pas, tidak bikin menggigil. Kru selalu menyapa saat naik dan turun. Bakal langganan terus kalau ke Solo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>Bayu Pratama</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>PO Rosalia Indah</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Solo (Palur)</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>First Class Double Decker</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I72" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Sleeper</t>
+        </is>
+      </c>
+      <c r="J72" s="3" t="inlineStr">
+        <is>
+          <t>First Class serasa naik pesawat bisnis</t>
+        </is>
+      </c>
+      <c r="K72" s="3" t="inlineStr">
+        <is>
+          <t>Kursi elektrik bisa diatur pijatan getarnya. Ada layar hiburan pribadi dan sandal hotel gratis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>Joko Susilo</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>PO Rosalia Indah</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Kampung Rambutan) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>Super Top Double Decker</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
+          <t>Ketepatan Waktu</t>
+        </is>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>Waktu kedatangan di Bungurasih sesuai jadwal</t>
+        </is>
+      </c>
+      <c r="K73" s="3" t="inlineStr">
+        <is>
+          <t>Meskipun keluar terminal agak padat, di Tol Cipali dan Semarang supir ngebut halus dan tiba jam 06:00 pagi pas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>Siti Aminah</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>PO Sinar Jaya</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>Suite Class Sleeper</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I74" s="3" t="inlineStr">
+        <is>
+          <t>Harga &amp; Kenyamanan</t>
+        </is>
+      </c>
+      <c r="J74" s="3" t="inlineStr">
+        <is>
+          <t>Sleeper bus paling ramah kantong di Indonesia</t>
+        </is>
+      </c>
+      <c r="K74" s="3" t="inlineStr">
+        <is>
+          <t>Harga tiket Suite Class cuma Rp 400 ribuan tapi sudah dapat kamar pod sleeper privat. Tirai penutup rapat jadi tidak canggung. Sangat hemat dibanding sleeper bus lain yang 600 ribuan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>Rian Kurniawan</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>PO Sinar Jaya</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Kampung Rambutan) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>Executive Legrest</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
+          <t>Ketepatan Waktu</t>
+        </is>
+      </c>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>Disiplin jam berangkat dari terminal</t>
+        </is>
+      </c>
+      <c r="K75" s="3" t="inlineStr">
+        <is>
+          <t>Sinar Jaya terkenal tidak suka ngetem lama-lama di agen. Jam 07:00 terjadwal langsung berangkat. Tiba di Solo tepat waktu sore jam 15:30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>Fajar Nugroho</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>PO Sinar Jaya</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>Suite Class Sleeper</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I76" s="3" t="inlineStr">
+        <is>
+          <t>Kenyamanan Kabin</t>
+        </is>
+      </c>
+      <c r="J76" s="3" t="inlineStr">
+        <is>
+          <t>Kabin dek atas agak sempit ruang kepalanya</t>
+        </is>
+      </c>
+      <c r="K76" s="3" t="inlineStr">
+        <is>
+          <t>Untuk tidur lurus sangat nyaman, tapi kalau duduk tegak di kasur atas kepala sedikit mentok plafon. Tapi untuk harga segini sangat memuaskan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>Wahyu Hidayat</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>PO Sinar Jaya</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Kalideres) → Semarang (Terboyo / Krapyak)</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>Executive Legrest</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
+          <t>Ekonomis</t>
+        </is>
+      </c>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>Pilihan terbaik untuk pulang kampung hemat</t>
+        </is>
+      </c>
+      <c r="K77" s="3" t="inlineStr">
+        <is>
+          <t>Tiket Eksekutif cuma Rp 230 ribuan ke Semarang. Kursi legrest cukup empuk, AC dingin, supir mengemudi dengan eco-driving tenang.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>Endang Supriyati</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>PO Sinar Jaya</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>Suite Class Sleeper</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I78" s="3" t="inlineStr">
+        <is>
+          <t>Kebersihan Kabin</t>
+        </is>
+      </c>
+      <c r="J78" s="3" t="inlineStr">
+        <is>
+          <t>Sprei dan sarung bantal diganti baru</t>
+        </is>
+      </c>
+      <c r="K78" s="3" t="inlineStr">
+        <is>
+          <t>Masuk kabin sleeper tercium wangi deterjen bersih. Dikasih sandal plastik untuk ke toilet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>Bagus Wicaksono</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>PO Sinar Jaya</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Solo (Tirtonadi)</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>Executive Legrest</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I79" s="3" t="inlineStr">
+        <is>
+          <t>Makan Rest Area</t>
+        </is>
+      </c>
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t>Servis makan standar tapi cukup mengenyangkan</t>
+        </is>
+      </c>
+      <c r="K79" s="3" t="inlineStr">
+        <is>
+          <t>Resto rekanan di Tol Cipali cukup bersih, menu nasi rendang ayam standar. Jangan berharap mewah, tapi sebanding harga tiket.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>Indra Permana</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>RedBus ID (Verified Ticket)</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>PO Sinar Jaya</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Kampung Rambutan) → Surabaya (Bungurasih)</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>Suite Class Sleeper</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I80" s="3" t="inlineStr">
+        <is>
+          <t>Ketepatan Waktu</t>
+        </is>
+      </c>
+      <c r="J80" s="3" t="inlineStr">
+        <is>
+          <t>Jam tiba subuh pas untuk jemputan</t>
+        </is>
+      </c>
+      <c r="K80" s="3" t="inlineStr">
+        <is>
+          <t>Berangkat sore jam 16:30 dari Rambutan, tiba jam 04:45 di Bungurasih. Sopir tidak ugal-ugalan tapi jalannya stabil 85 km/jam.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>Dedi Mulyadi Fan</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>Traveloka Verified Passenger</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>PO Sinar Jaya</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>Jakarta (Pulo Gebang) → Semarang (Krapyak)</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>Executive Legrest</t>
+        </is>
+      </c>
+      <c r="G81" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>POSITIF</t>
+        </is>
+      </c>
+      <c r="I81" s="3" t="inlineStr">
+        <is>
+          <t>Pelayanan Kru</t>
+        </is>
+      </c>
+      <c r="J81" s="3" t="inlineStr">
+        <is>
+          <t>Kondektur cekatan dan ramah</t>
+        </is>
+      </c>
+      <c r="K81" s="3" t="inlineStr">
+        <is>
+          <t>Barang bagasi ditandai spidol rapi. Penurunan di Krapyak tidak ribet.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -478,9 +4963,8 @@
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="32" customWidth="1" min="11" max="11"/>
     <col width="33" customWidth="1" min="12" max="12"/>
-    <col width="60" customWidth="1" min="13" max="13"/>
-    <col width="60" customWidth="1" min="14" max="14"/>
-    <col width="60" customWidth="1" min="15" max="15"/>
+    <col width="70" customWidth="1" min="13" max="13"/>
+    <col width="70" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -554,11 +5038,6 @@
           <t>Poin Perhatian Penumpang</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
-        <is>
-          <t>Kutipan Ulasan Riil</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -611,11 +5090,6 @@
           <t>Harga tiket kelas atas, kuota kursi terbatas (wajib pesan jauh hari sebelum keberangkatan).</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>Naik dari Pondok Pinang ke Malang tidur nyenyak banget. Pod sleeper kedap suara, toilet bersih, makanan enak. | Pramugara ramah, dikasih bantal selimut tebal dan wangi. Tiba di Surabaya on time sesuai jadwal.</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -668,11 +5142,6 @@
           <t>Kursi deretan paling belakang terasa sedikit lebih kaku di jalan tol bergelombang.</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
-        <is>
-          <t>Desain interior elegan dan bersih. Driver bawa busnya sangat halus di Tol Cipali. | Kelas President benar-benar bikin badan segar pas sampai tujuan. Tidak capek sama sekali.</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -725,11 +5194,6 @@
           <t>Waktu istirahat makan di rest area sangat ketat sesuai jadwal operasional.</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
-        <is>
-          <t>Bus hijau kesayangan. Mesin halus, supir tidak ugal-ugalan tapi jalan tetap taktis dan on-time. | Kabin wangi, leg rest luas, AC dingin stabil sepanjang perjalanan Jakarta - Surabaya.</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -782,11 +5246,6 @@
           <t>Titik agen penjemputan arteri cukup banyak sehingga waktu tempuh sebelum masuk tol utama relatif panjang.</t>
         </is>
       </c>
-      <c r="O5" s="3" t="inlineStr">
-        <is>
-          <t>Pelayanan pramugari seperti di pesawat, dibantu bawain barang. Makan malam di Resto Rosin mantap. | Armada Double Decker tingkat bawahnya sangat nyaman. Rekomendasi buat perjalanan keluarga.</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -839,11 +5298,6 @@
           <t>Kondisi fisik armada bervariasi antara bus rilis baru dengan unit yang lebih lama.</t>
         </is>
       </c>
-      <c r="O6" s="3" t="inlineStr">
-        <is>
-          <t>Tiketnya terjangkau dan keberangkatan tepat waktu dari pul Pondok Pinang. | Supir bawa bus cepat sampai, cocok buat yang butuh sampai pagi-pagi sekali di terminal tujuan.</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -896,11 +5350,6 @@
           <t>Gaya berkendara di tol relatif agresif (bus malam cepat), kurang disarankan bagi penumpang yang mudah mual.</t>
         </is>
       </c>
-      <c r="O7" s="3" t="inlineStr">
-        <is>
-          <t>Mantap Menara Kudus, jam 4 subuh sudah mendarat di Solo. Servis makan soto ayamnya juara. | Bus banter tapi supir berpengalaman tahu medan tol Trans-Jawa. Kru ramah saat menaikkan bagasi.</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -953,11 +5402,6 @@
           <t>Kecepatan maksimal dibatasi limiter mesin (85-90 km/jam) sehingga waktu jelajah sedikit lebih lambat.</t>
         </is>
       </c>
-      <c r="O8" s="3" t="inlineStr">
-        <is>
-          <t>Pilihan paling aman dan tenang kalau bawa orang tua atau anak kecil. Supir bawa bus kalem. | Suite class-nya murah dibanding PO lain tapi tetap dapat fasilitas kasur privat yang nyaman.</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1010,11 +5454,6 @@
           <t>Pul agen di wilayah timur Jakarta cukup padat saat jam sibuk sore.</t>
         </is>
       </c>
-      <c r="O9" s="3" t="inlineStr">
-        <is>
-          <t>Naik Double Decker Agra Mas ke Madiun nyaman sekali, suspensi empuk dan toilet bersih. | Servis makan di RM Kendil Mas enak, kru komunikatif saat pembagian snack keberangkatan.</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1067,11 +5506,6 @@
           <t>Tiket kelas Luxury Sleeper cepat ludes, terutama tujuan Tulungagung dan Blitar.</t>
         </is>
       </c>
-      <c r="O10" s="3" t="inlineStr">
-        <is>
-          <t>Kuda oranye andalan sejak dulu. Kursi sleepernya empuk, ac sejuk, dan supir sangat tertib. | Perjalanan malam tidur pulas. Fasilitas lengkap dan tepat waktu sampai terminal.</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1122,11 +5556,6 @@
       <c r="N11" s="3" t="inlineStr">
         <is>
           <t>Frekuensi jadwal harian lebih terfokus dibanding operator raksasa lainnya.</t>
-        </is>
-      </c>
-      <c r="O11" s="3" t="inlineStr">
-        <is>
-          <t>Khas PO legendaris Kudus, kenyamanan mesin Mercy dan Scania tidak pernah bohong. | Kru berseragam rapi, keberangkatan dari agen tepat waktu, kabin tidak bising.</t>
         </is>
       </c>
     </row>
@@ -1135,7 +5564,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2325,7 +6754,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2839,7 +7268,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -35447,7 +39876,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>